<commit_message>
Worked on Animal.py class. Cleaned up Scent class a little bit. Modified .gitignore and Milestones-for-thesis
</commit_message>
<xml_diff>
--- a/documents/Milestones-for-thesis.xlsx
+++ b/documents/Milestones-for-thesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\cisc-699\final-project\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E15F7C3D-44DC-40AD-810B-CC7D8B43FE03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1D0FB1E-B1E0-4680-81D2-F514A3B9B209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
   </bookViews>
@@ -220,7 +220,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d;@"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -235,22 +235,8 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF9C5700"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="14"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF9C5700"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -271,6 +257,13 @@
     <font>
       <b/>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -310,13 +303,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
   </fills>
@@ -456,45 +450,42 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Neutral" xfId="1" builtinId="28"/>
+    <cellStyle name="20% - Accent1" xfId="1" builtinId="30"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
@@ -866,696 +857,697 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8008939-BF20-4CB8-B4D2-4F26019E5DA8}">
-  <dimension ref="B1:D66"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:D67"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.28515625" style="7" customWidth="1"/>
-    <col min="2" max="2" width="50" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="7"/>
+    <col min="1" max="1" width="2.28515625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="50" style="5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" style="5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:4" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="8" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="23" t="s">
+      <c r="B3" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="25">
+      <c r="D3" s="22">
         <v>46158</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B4" s="12" t="s">
+    <row r="4" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="14">
+      <c r="D4" s="12">
         <v>46156</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B5" s="15" t="s">
+    <row r="5" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="17">
+      <c r="D5" s="15">
         <v>46157</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B6" s="15" t="s">
+    <row r="6" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="16" t="s">
+      <c r="C6" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="16">
         <v>46158</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B7" s="15"/>
-      <c r="C7" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="17"/>
-    </row>
-    <row r="8" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="19"/>
-      <c r="C8" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" s="21"/>
-    </row>
-    <row r="9" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="5" t="s">
+    <row r="7" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="13"/>
+      <c r="C7" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="15"/>
+    </row>
+    <row r="8" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="17"/>
+      <c r="C8" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="19"/>
+    </row>
+    <row r="9" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9" s="26">
+      <c r="C9" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="23">
         <v>46165</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B10" s="12" t="s">
+    <row r="10" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="C10" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" s="22">
+      <c r="C10" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="20">
         <v>46160</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B11" s="15" t="s">
+    <row r="11" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="C11" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11" s="17">
+      <c r="C11" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="15">
         <v>46164</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B12" s="15" t="s">
+    <row r="12" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" s="17">
+      <c r="C12" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="15">
         <v>46165</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B13" s="15" t="s">
+    <row r="13" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="C13" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D13" s="17">
+      <c r="C13" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="15">
         <v>46165</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="19"/>
-      <c r="C14" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14" s="21"/>
+    <row r="14" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="17"/>
+      <c r="C14" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="19"/>
     </row>
     <row r="15" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="27" t="s">
         <v>5</v>
       </c>
-      <c r="C15" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D15" s="27">
+      <c r="C15" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="24">
         <v>46172</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B16" s="12" t="s">
+    <row r="16" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D16" s="22">
+      <c r="C16" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="20">
         <v>46168</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B17" s="15" t="s">
+    <row r="17" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D17" s="17">
+      <c r="C17" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="15">
         <v>46168</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B18" s="15" t="s">
+    <row r="18" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B18" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D18" s="17">
+      <c r="C18" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="15">
         <v>46170</v>
       </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B19" s="15" t="s">
+    <row r="19" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D19" s="17">
+      <c r="C19" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="15">
         <v>46171</v>
       </c>
     </row>
-    <row r="20" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="19" t="s">
+    <row r="20" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="D20" s="21">
+      <c r="C20" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="19">
         <v>46172</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="C21" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D21" s="28">
+      <c r="C21" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="25">
         <v>46186</v>
       </c>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B22" s="12" t="s">
+    <row r="22" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C22" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D22" s="22">
+      <c r="C22" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="20">
         <v>46177</v>
       </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B23" s="15" t="s">
+    <row r="23" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="C23" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D23" s="17">
+      <c r="C23" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" s="15">
         <v>46184</v>
       </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B24" s="15" t="s">
+    <row r="24" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B24" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="C24" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D24" s="17">
+      <c r="C24" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D24" s="15">
         <v>46185</v>
       </c>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B25" s="15" t="s">
+    <row r="25" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B25" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C25" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D25" s="17">
+      <c r="C25" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D25" s="15">
         <v>46185</v>
       </c>
     </row>
-    <row r="26" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="19" t="s">
+    <row r="26" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="C26" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="D26" s="21">
+      <c r="C26" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="19">
         <v>46186</v>
       </c>
     </row>
     <row r="27" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="C27" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D27" s="28">
+      <c r="C27" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="25">
         <v>46200</v>
       </c>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B28" s="12" t="s">
+    <row r="28" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C28" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D28" s="22">
+      <c r="C28" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="20">
         <v>46193</v>
       </c>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B29" s="15" t="s">
+    <row r="29" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="C29" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D29" s="17">
+      <c r="C29" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="15">
         <v>46197</v>
       </c>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B30" s="15" t="s">
+    <row r="30" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C30" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D30" s="17">
+      <c r="C30" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D30" s="15">
         <v>46199</v>
       </c>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B31" s="19" t="s">
+    <row r="31" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="C31" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D31" s="17">
+      <c r="C31" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="15">
         <v>46200</v>
       </c>
     </row>
-    <row r="32" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="19"/>
-      <c r="C32" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="D32" s="21"/>
-    </row>
-    <row r="33" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="5" t="s">
+    <row r="32" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="17"/>
+      <c r="C32" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="19"/>
+    </row>
+    <row r="33" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="C33" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D33" s="28">
+      <c r="C33" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" s="25">
         <v>46214</v>
       </c>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B34" s="12" t="s">
+    <row r="34" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="C34" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D34" s="22">
+      <c r="C34" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34" s="20">
         <v>46203</v>
       </c>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B35" s="15" t="s">
+    <row r="35" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="C35" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D35" s="17">
+      <c r="C35" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35" s="15">
         <v>46212</v>
       </c>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B36" s="15" t="s">
+    <row r="36" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C36" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D36" s="17">
+      <c r="C36" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="15">
         <v>46213</v>
       </c>
     </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B37" s="15" t="s">
+    <row r="37" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C37" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D37" s="17">
+      <c r="C37" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37" s="15">
         <v>46213</v>
       </c>
     </row>
-    <row r="38" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B38" s="19" t="s">
+    <row r="38" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C38" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="D38" s="21">
+      <c r="C38" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="19">
         <v>46214</v>
       </c>
     </row>
-    <row r="39" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="19" t="s">
+    <row r="39" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="C39" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="D39" s="21">
+      <c r="C39" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D39" s="19">
         <v>46214</v>
       </c>
     </row>
-    <row r="40" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="5" t="s">
+    <row r="40" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="C40" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D40" s="28">
+      <c r="C40" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D40" s="25">
         <v>46235</v>
       </c>
     </row>
-    <row r="41" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B41" s="12" t="s">
+    <row r="41" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="C41" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D41" s="22">
+      <c r="C41" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D41" s="20">
         <v>46227</v>
       </c>
     </row>
-    <row r="42" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B42" s="15" t="s">
+    <row r="42" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B42" s="27" t="s">
         <v>39</v>
       </c>
-      <c r="C42" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D42" s="17">
+      <c r="C42" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D42" s="15">
         <v>46232</v>
       </c>
     </row>
-    <row r="43" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B43" s="15" t="s">
+    <row r="43" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="C43" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D43" s="17">
+      <c r="C43" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D43" s="15">
         <v>46232</v>
       </c>
     </row>
-    <row r="44" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B44" s="15" t="s">
+    <row r="44" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B44" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C44" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D44" s="17">
+      <c r="C44" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D44" s="15">
         <v>46233</v>
       </c>
     </row>
-    <row r="45" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B45" s="15" t="s">
+    <row r="45" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B45" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="C45" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D45" s="17">
+      <c r="C45" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D45" s="15">
         <v>46233</v>
       </c>
     </row>
-    <row r="46" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B46" s="15" t="s">
+    <row r="46" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C46" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D46" s="17">
+      <c r="C46" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D46" s="15">
         <v>46234</v>
       </c>
     </row>
-    <row r="47" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B47" s="15" t="s">
+    <row r="47" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B47" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="C47" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D47" s="17">
+      <c r="C47" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D47" s="15">
         <v>46235</v>
       </c>
     </row>
-    <row r="48" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="19" t="s">
+    <row r="48" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B48" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C48" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="D48" s="21">
+      <c r="C48" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D48" s="19">
         <v>46235</v>
       </c>
     </row>
-    <row r="49" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="5" t="s">
+    <row r="49" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B49" s="27" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D49" s="28">
+      <c r="C49" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D49" s="25">
         <v>46239</v>
       </c>
     </row>
-    <row r="50" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B50" s="12" t="s">
+    <row r="50" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B50" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="C50" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D50" s="22">
+      <c r="C50" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D50" s="20">
         <v>46237</v>
       </c>
     </row>
-    <row r="51" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B51" s="15" t="s">
+    <row r="51" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B51" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="C51" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D51" s="17">
+      <c r="C51" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D51" s="15">
         <v>46238</v>
       </c>
     </row>
-    <row r="52" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B52" s="15" t="s">
+    <row r="52" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B52" s="27" t="s">
         <v>30</v>
       </c>
-      <c r="C52" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D52" s="17">
+      <c r="C52" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D52" s="15">
         <v>46239</v>
       </c>
     </row>
-    <row r="53" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B53" s="15"/>
-      <c r="C53" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D53" s="17"/>
-    </row>
-    <row r="54" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B54" s="19"/>
-      <c r="C54" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="D54" s="21"/>
-    </row>
-    <row r="55" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="5" t="s">
+    <row r="53" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B53" s="27"/>
+      <c r="C53" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D53" s="15"/>
+    </row>
+    <row r="54" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B54" s="27"/>
+      <c r="C54" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D54" s="19"/>
+    </row>
+    <row r="55" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B55" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="C55" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D55" s="28">
+      <c r="C55" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D55" s="25">
         <v>46242</v>
       </c>
     </row>
-    <row r="56" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B56" s="12" t="s">
+    <row r="56" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B56" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="C56" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D56" s="22">
+      <c r="C56" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D56" s="20">
         <v>46240</v>
       </c>
     </row>
-    <row r="57" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B57" s="15" t="s">
+    <row r="57" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B57" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="C57" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D57" s="17">
+      <c r="C57" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D57" s="15">
         <v>46241</v>
       </c>
     </row>
-    <row r="58" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B58" s="15" t="s">
+    <row r="58" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B58" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="C58" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D58" s="17">
+      <c r="C58" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D58" s="15">
         <v>46242</v>
       </c>
     </row>
-    <row r="59" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B59" s="15" t="s">
+    <row r="59" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B59" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="C59" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D59" s="17">
+      <c r="C59" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D59" s="15">
         <v>46242</v>
       </c>
     </row>
-    <row r="60" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="19"/>
-      <c r="C60" s="20" t="s">
-        <v>14</v>
-      </c>
-      <c r="D60" s="21"/>
-    </row>
-    <row r="61" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="5" t="s">
+    <row r="60" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B60" s="27"/>
+      <c r="C60" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="D60" s="19"/>
+    </row>
+    <row r="61" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B61" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="C61" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D61" s="26">
+      <c r="C61" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D61" s="23">
         <v>46249</v>
       </c>
     </row>
-    <row r="62" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B62" s="12" t="s">
+    <row r="62" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B62" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="C62" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D62" s="22">
+      <c r="C62" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D62" s="20">
         <v>46249</v>
       </c>
     </row>
-    <row r="63" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B63" s="15" t="s">
+    <row r="63" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B63" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="C63" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D63" s="17">
+      <c r="C63" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D63" s="15">
         <v>46249</v>
       </c>
     </row>
-    <row r="64" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B64" s="15" t="s">
+    <row r="64" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B64" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="C64" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D64" s="17">
+      <c r="C64" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D64" s="15">
         <v>46249</v>
       </c>
     </row>
-    <row r="65" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B65" s="15"/>
-      <c r="C65" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D65" s="17"/>
-    </row>
-    <row r="66" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B66" s="15"/>
-      <c r="C66" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D66" s="17"/>
-    </row>
+    <row r="65" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B65" s="13"/>
+      <c r="C65" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D65" s="15"/>
+    </row>
+    <row r="66" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B66" s="13"/>
+      <c r="C66" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D66" s="15"/>
+    </row>
+    <row r="67" spans="2:4" collapsed="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Code refactor. Created a more general version of scent_search. Moved scent_search into the Scent.py
</commit_message>
<xml_diff>
--- a/documents/Milestones-for-thesis.xlsx
+++ b/documents/Milestones-for-thesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\cisc-699\final-project\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1D0FB1E-B1E0-4680-81D2-F514A3B9B209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8C9E7C5-5B7E-4820-9F89-5C1913A6DDA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
   </bookViews>
@@ -964,7 +964,7 @@
         <v>48</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D11" s="15">
         <v>46164</v>
@@ -975,7 +975,7 @@
         <v>49</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D12" s="15">
         <v>46165</v>
@@ -986,7 +986,7 @@
         <v>55</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D13" s="15">
         <v>46165</v>

</xml_diff>

<commit_message>
Finished Animal and Scent class. Added class level self testing.
</commit_message>
<xml_diff>
--- a/documents/Milestones-for-thesis.xlsx
+++ b/documents/Milestones-for-thesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\cisc-699\final-project\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8C9E7C5-5B7E-4820-9F89-5C1913A6DDA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F37D0D9A-35E4-4406-A16D-57CAEFB593B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
   </bookViews>
@@ -942,13 +942,13 @@
         <v>4</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D9" s="23">
         <v>46165</v>
       </c>
     </row>
-    <row r="10" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B10" s="10" t="s">
         <v>47</v>
       </c>
@@ -959,7 +959,7 @@
         <v>46160</v>
       </c>
     </row>
-    <row r="11" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B11" s="13" t="s">
         <v>48</v>
       </c>
@@ -970,36 +970,36 @@
         <v>46164</v>
       </c>
     </row>
-    <row r="12" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B12" s="13" t="s">
         <v>49</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D12" s="15">
         <v>46165</v>
       </c>
     </row>
-    <row r="13" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B13" s="13" t="s">
         <v>55</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D13" s="15">
         <v>46165</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="17"/>
       <c r="C14" s="18" t="s">
         <v>14</v>
       </c>
       <c r="D14" s="19"/>
     </row>
-    <row r="15" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="27" t="s">
         <v>5</v>
       </c>
@@ -1142,7 +1142,7 @@
         <v>46200</v>
       </c>
     </row>
-    <row r="28" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B28" s="10" t="s">
         <v>7</v>
       </c>
@@ -1153,7 +1153,7 @@
         <v>46193</v>
       </c>
     </row>
-    <row r="29" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B29" s="13" t="s">
         <v>8</v>
       </c>
@@ -1164,7 +1164,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="30" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B30" s="13" t="s">
         <v>9</v>
       </c>
@@ -1175,7 +1175,7 @@
         <v>46199</v>
       </c>
     </row>
-    <row r="31" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B31" s="17" t="s">
         <v>56</v>
       </c>
@@ -1186,14 +1186,14 @@
         <v>46200</v>
       </c>
     </row>
-    <row r="32" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="17"/>
       <c r="C32" s="18" t="s">
         <v>14</v>
       </c>
       <c r="D32" s="19"/>
     </row>
-    <row r="33" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="27" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Map class basic outline with getters.
</commit_message>
<xml_diff>
--- a/documents/Milestones-for-thesis.xlsx
+++ b/documents/Milestones-for-thesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\cisc-699\final-project\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F37D0D9A-35E4-4406-A16D-57CAEFB593B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38DA3D82-42E4-4071-8C84-557618D4A4B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="58">
   <si>
     <t>Task</t>
   </si>
@@ -211,6 +211,9 @@
   </si>
   <si>
     <t>class testers</t>
+  </si>
+  <si>
+    <t>getters</t>
   </si>
 </sst>
 </file>
@@ -314,7 +317,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -447,12 +450,40 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -482,7 +513,13 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="7" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="10" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="20% - Accent1" xfId="1" builtinId="30"/>
@@ -857,7 +894,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8008939-BF20-4CB8-B4D2-4F26019E5DA8}">
-  <dimension ref="B1:D67"/>
+  <dimension ref="B1:D66"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.28515625" style="5" customWidth="1"/>
@@ -890,7 +927,7 @@
         <v>46158</v>
       </c>
     </row>
-    <row r="4" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B4" s="10" t="s">
         <v>3</v>
       </c>
@@ -901,7 +938,7 @@
         <v>46156</v>
       </c>
     </row>
-    <row r="5" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B5" s="13" t="s">
         <v>45</v>
       </c>
@@ -912,7 +949,7 @@
         <v>46157</v>
       </c>
     </row>
-    <row r="6" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B6" s="13" t="s">
         <v>46</v>
       </c>
@@ -923,22 +960,22 @@
         <v>46158</v>
       </c>
     </row>
-    <row r="7" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B7" s="13"/>
       <c r="C7" s="14" t="s">
         <v>14</v>
       </c>
       <c r="D7" s="15"/>
     </row>
-    <row r="8" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="17"/>
       <c r="C8" s="18" t="s">
         <v>14</v>
       </c>
       <c r="D8" s="19"/>
     </row>
-    <row r="9" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="27" t="s">
+    <row r="9" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="32" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="9" t="s">
@@ -948,7 +985,7 @@
         <v>46165</v>
       </c>
     </row>
-    <row r="10" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B10" s="10" t="s">
         <v>47</v>
       </c>
@@ -959,7 +996,7 @@
         <v>46160</v>
       </c>
     </row>
-    <row r="11" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B11" s="13" t="s">
         <v>48</v>
       </c>
@@ -970,7 +1007,7 @@
         <v>46164</v>
       </c>
     </row>
-    <row r="12" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B12" s="13" t="s">
         <v>49</v>
       </c>
@@ -981,7 +1018,7 @@
         <v>46165</v>
       </c>
     </row>
-    <row r="13" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B13" s="13" t="s">
         <v>55</v>
       </c>
@@ -992,19 +1029,19 @@
         <v>46165</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="17"/>
       <c r="C14" s="18" t="s">
         <v>14</v>
       </c>
       <c r="D14" s="19"/>
     </row>
-    <row r="15" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="27" t="s">
+    <row r="15" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="32" t="s">
         <v>5</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D15" s="24">
         <v>46172</v>
@@ -1015,7 +1052,7 @@
         <v>19</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D16" s="20">
         <v>46168</v>
@@ -1023,10 +1060,10 @@
     </row>
     <row r="17" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B17" s="13" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D17" s="15">
         <v>46168</v>
@@ -1037,7 +1074,7 @@
         <v>37</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D18" s="15">
         <v>46170</v>
@@ -1066,7 +1103,7 @@
       </c>
     </row>
     <row r="21" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="27" t="s">
+      <c r="B21" s="32" t="s">
         <v>6</v>
       </c>
       <c r="C21" s="9" t="s">
@@ -1132,7 +1169,7 @@
       </c>
     </row>
     <row r="27" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="27" t="s">
+      <c r="B27" s="32" t="s">
         <v>18</v>
       </c>
       <c r="C27" s="9" t="s">
@@ -1194,7 +1231,7 @@
       <c r="D32" s="19"/>
     </row>
     <row r="33" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="27" t="s">
+      <c r="B33" s="32" t="s">
         <v>10</v>
       </c>
       <c r="C33" s="9" t="s">
@@ -1204,7 +1241,7 @@
         <v>46214</v>
       </c>
     </row>
-    <row r="34" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B34" s="10" t="s">
         <v>47</v>
       </c>
@@ -1215,7 +1252,7 @@
         <v>46203</v>
       </c>
     </row>
-    <row r="35" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B35" s="13" t="s">
         <v>28</v>
       </c>
@@ -1226,7 +1263,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="36" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B36" s="13" t="s">
         <v>22</v>
       </c>
@@ -1237,7 +1274,7 @@
         <v>46213</v>
       </c>
     </row>
-    <row r="37" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B37" s="13" t="s">
         <v>23</v>
       </c>
@@ -1248,7 +1285,7 @@
         <v>46213</v>
       </c>
     </row>
-    <row r="38" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B38" s="17" t="s">
         <v>24</v>
       </c>
@@ -1259,7 +1296,7 @@
         <v>46214</v>
       </c>
     </row>
-    <row r="39" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B39" s="17" t="s">
         <v>55</v>
       </c>
@@ -1270,19 +1307,19 @@
         <v>46214</v>
       </c>
     </row>
-    <row r="40" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="27" t="s">
+    <row r="40" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="33" t="s">
         <v>36</v>
       </c>
-      <c r="C40" s="9" t="s">
+      <c r="C40" s="28" t="s">
         <v>14</v>
       </c>
       <c r="D40" s="25">
         <v>46235</v>
       </c>
     </row>
-    <row r="41" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="27" t="s">
+    <row r="41" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B41" s="29" t="s">
         <v>33</v>
       </c>
       <c r="C41" s="11" t="s">
@@ -1292,7 +1329,7 @@
         <v>46227</v>
       </c>
     </row>
-    <row r="42" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B42" s="27" t="s">
         <v>39</v>
       </c>
@@ -1303,7 +1340,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="43" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B43" s="27" t="s">
         <v>50</v>
       </c>
@@ -1314,7 +1351,7 @@
         <v>46232</v>
       </c>
     </row>
-    <row r="44" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B44" s="27" t="s">
         <v>27</v>
       </c>
@@ -1325,7 +1362,7 @@
         <v>46233</v>
       </c>
     </row>
-    <row r="45" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B45" s="27" t="s">
         <v>40</v>
       </c>
@@ -1336,7 +1373,7 @@
         <v>46233</v>
       </c>
     </row>
-    <row r="46" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B46" s="27" t="s">
         <v>25</v>
       </c>
@@ -1347,7 +1384,7 @@
         <v>46234</v>
       </c>
     </row>
-    <row r="47" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B47" s="27" t="s">
         <v>34</v>
       </c>
@@ -1358,8 +1395,8 @@
         <v>46235</v>
       </c>
     </row>
-    <row r="48" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="27" t="s">
+    <row r="48" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B48" s="31" t="s">
         <v>26</v>
       </c>
       <c r="C48" s="18" t="s">
@@ -1369,19 +1406,19 @@
         <v>46235</v>
       </c>
     </row>
-    <row r="49" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="27" t="s">
+    <row r="49" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B49" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="28" t="s">
         <v>14</v>
       </c>
       <c r="D49" s="25">
         <v>46239</v>
       </c>
     </row>
-    <row r="50" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="27" t="s">
+    <row r="50" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B50" s="29" t="s">
         <v>35</v>
       </c>
       <c r="C50" s="11" t="s">
@@ -1391,7 +1428,7 @@
         <v>46237</v>
       </c>
     </row>
-    <row r="51" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B51" s="27" t="s">
         <v>29</v>
       </c>
@@ -1402,7 +1439,7 @@
         <v>46238</v>
       </c>
     </row>
-    <row r="52" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B52" s="27" t="s">
         <v>30</v>
       </c>
@@ -1413,33 +1450,33 @@
         <v>46239</v>
       </c>
     </row>
-    <row r="53" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B53" s="27"/>
       <c r="C53" s="14" t="s">
         <v>14</v>
       </c>
       <c r="D53" s="15"/>
     </row>
-    <row r="54" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B54" s="27"/>
+    <row r="54" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B54" s="31"/>
       <c r="C54" s="18" t="s">
         <v>14</v>
       </c>
       <c r="D54" s="19"/>
     </row>
-    <row r="55" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="27" t="s">
+    <row r="55" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B55" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="C55" s="9" t="s">
+      <c r="C55" s="28" t="s">
         <v>14</v>
       </c>
       <c r="D55" s="25">
         <v>46242</v>
       </c>
     </row>
-    <row r="56" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="27" t="s">
+    <row r="56" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="B56" s="29" t="s">
         <v>42</v>
       </c>
       <c r="C56" s="11" t="s">
@@ -1449,7 +1486,7 @@
         <v>46240</v>
       </c>
     </row>
-    <row r="57" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B57" s="27" t="s">
         <v>31</v>
       </c>
@@ -1460,7 +1497,7 @@
         <v>46241</v>
       </c>
     </row>
-    <row r="58" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B58" s="27" t="s">
         <v>43</v>
       </c>
@@ -1471,7 +1508,7 @@
         <v>46242</v>
       </c>
     </row>
-    <row r="59" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B59" s="27" t="s">
         <v>32</v>
       </c>
@@ -1482,25 +1519,25 @@
         <v>46242</v>
       </c>
     </row>
-    <row r="60" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B60" s="27"/>
+    <row r="60" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B60" s="31"/>
       <c r="C60" s="18" t="s">
         <v>14</v>
       </c>
       <c r="D60" s="19"/>
     </row>
-    <row r="61" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="27" t="s">
+    <row r="61" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B61" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="C61" s="9" t="s">
+      <c r="C61" s="28" t="s">
         <v>14</v>
       </c>
       <c r="D61" s="23">
         <v>46249</v>
       </c>
     </row>
-    <row r="62" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B62" s="10" t="s">
         <v>52</v>
       </c>
@@ -1511,7 +1548,7 @@
         <v>46249</v>
       </c>
     </row>
-    <row r="63" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B63" s="13" t="s">
         <v>53</v>
       </c>
@@ -1522,7 +1559,7 @@
         <v>46249</v>
       </c>
     </row>
-    <row r="64" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B64" s="13" t="s">
         <v>54</v>
       </c>
@@ -1533,21 +1570,20 @@
         <v>46249</v>
       </c>
     </row>
-    <row r="65" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B65" s="13"/>
       <c r="C65" s="14" t="s">
         <v>14</v>
       </c>
       <c r="D65" s="15"/>
     </row>
-    <row r="66" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B66" s="13"/>
       <c r="C66" s="14" t="s">
         <v>14</v>
       </c>
       <c r="D66" s="15"/>
     </row>
-    <row r="67" spans="2:4" collapsed="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
readability update for readme and documents
</commit_message>
<xml_diff>
--- a/documents/Milestones-for-thesis.xlsx
+++ b/documents/Milestones-for-thesis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\cisc-699\final-project\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4400027-4155-49D3-B2EB-00346B50DFF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18EE3AF3-934C-4FF0-8644-7A8E2B91955B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3465" yWindow="3465" windowWidth="21600" windowHeight="11385" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
   </bookViews>
   <sheets>
     <sheet name="Milestones" sheetId="1" r:id="rId1"/>
@@ -1107,7 +1107,7 @@
         <v>6</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D21" s="25">
         <v>46186</v>
@@ -1118,7 +1118,7 @@
         <v>38</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D22" s="20">
         <v>46177</v>
@@ -1129,7 +1129,7 @@
         <v>51</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D23" s="15">
         <v>46184</v>
@@ -1140,7 +1140,7 @@
         <v>20</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D24" s="15">
         <v>46185</v>
@@ -1151,7 +1151,7 @@
         <v>21</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D25" s="15">
         <v>46185</v>
@@ -1162,7 +1162,7 @@
         <v>50</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D26" s="19">
         <v>46186</v>

</xml_diff>

<commit_message>
compleated energy use and Animal class tester. Better pathfinding test needed.
</commit_message>
<xml_diff>
--- a/documents/Milestones-for-thesis.xlsx
+++ b/documents/Milestones-for-thesis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\cisc-699\final-project\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCBEC681-46E1-4248-B3B5-CC78C524CAE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9FFC76E-6B60-4289-A486-E06B7C60B7F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
+    <workbookView xWindow="3465" yWindow="3465" windowWidth="21600" windowHeight="11385" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
   </bookViews>
   <sheets>
     <sheet name="Milestones" sheetId="1" r:id="rId1"/>
@@ -1107,7 +1107,7 @@
         <v>6</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D21" s="25">
         <v>46186</v>
@@ -1140,7 +1140,7 @@
         <v>20</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D24" s="15">
         <v>46185</v>
@@ -1151,7 +1151,7 @@
         <v>21</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D25" s="15">
         <v>46185</v>
@@ -1162,7 +1162,7 @@
         <v>49</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D26" s="19">
         <v>46186</v>
@@ -1173,7 +1173,7 @@
         <v>18</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D27" s="25">
         <v>46200</v>
@@ -1184,7 +1184,7 @@
         <v>7</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D28" s="20">
         <v>46193</v>

</xml_diff>

<commit_message>
compleated energy use and Animal class tester. Better pathfinding test needed. (#4)
</commit_message>
<xml_diff>
--- a/documents/Milestones-for-thesis.xlsx
+++ b/documents/Milestones-for-thesis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\cisc-699\final-project\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCBEC681-46E1-4248-B3B5-CC78C524CAE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9FFC76E-6B60-4289-A486-E06B7C60B7F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
+    <workbookView xWindow="3465" yWindow="3465" windowWidth="21600" windowHeight="11385" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
   </bookViews>
   <sheets>
     <sheet name="Milestones" sheetId="1" r:id="rId1"/>
@@ -1107,7 +1107,7 @@
         <v>6</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D21" s="25">
         <v>46186</v>
@@ -1140,7 +1140,7 @@
         <v>20</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D24" s="15">
         <v>46185</v>
@@ -1151,7 +1151,7 @@
         <v>21</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D25" s="15">
         <v>46185</v>
@@ -1162,7 +1162,7 @@
         <v>49</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D26" s="19">
         <v>46186</v>
@@ -1173,7 +1173,7 @@
         <v>18</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D27" s="25">
         <v>46200</v>
@@ -1184,7 +1184,7 @@
         <v>7</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D28" s="20">
         <v>46193</v>

</xml_diff>

<commit_message>
current update for prey classes. Prey classes done need to build out class testers
</commit_message>
<xml_diff>
--- a/documents/Milestones-for-thesis.xlsx
+++ b/documents/Milestones-for-thesis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\cisc-699\final-project\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9FFC76E-6B60-4289-A486-E06B7C60B7F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE4088BA-BF56-43D3-88E1-D2F8B9EC6DE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3465" yWindow="3465" windowWidth="21600" windowHeight="11385" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
   </bookViews>
@@ -1047,7 +1047,7 @@
         <v>46172</v>
       </c>
     </row>
-    <row r="16" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B16" s="10" t="s">
         <v>19</v>
       </c>
@@ -1058,7 +1058,7 @@
         <v>46168</v>
       </c>
     </row>
-    <row r="17" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B17" s="13" t="s">
         <v>57</v>
       </c>
@@ -1069,7 +1069,7 @@
         <v>46168</v>
       </c>
     </row>
-    <row r="18" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B18" s="13" t="s">
         <v>37</v>
       </c>
@@ -1080,7 +1080,7 @@
         <v>46170</v>
       </c>
     </row>
-    <row r="19" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B19" s="13" t="s">
         <v>49</v>
       </c>
@@ -1091,7 +1091,7 @@
         <v>46171</v>
       </c>
     </row>
-    <row r="20" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="17" t="s">
         <v>55</v>
       </c>
@@ -1102,7 +1102,7 @@
         <v>46172</v>
       </c>
     </row>
-    <row r="21" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="32" t="s">
         <v>6</v>
       </c>
@@ -1173,7 +1173,7 @@
         <v>18</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D27" s="25">
         <v>46200</v>
@@ -1184,7 +1184,7 @@
         <v>7</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D28" s="20">
         <v>46193</v>
@@ -1195,7 +1195,7 @@
         <v>8</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D29" s="15">
         <v>46197</v>
@@ -1206,7 +1206,7 @@
         <v>9</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D30" s="15">
         <v>46199</v>
@@ -1217,7 +1217,7 @@
         <v>56</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D31" s="15">
         <v>46200</v>
@@ -1246,7 +1246,7 @@
         <v>47</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D34" s="20">
         <v>46203</v>

</xml_diff>

<commit_message>
start to predator class getters/setters
</commit_message>
<xml_diff>
--- a/documents/Milestones-for-thesis.xlsx
+++ b/documents/Milestones-for-thesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\cisc-699\final-project\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27036DF7-34BA-4C4B-B5C0-998D64350232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F26D26FD-4475-413E-AF1D-EA4759190F63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
   </bookViews>
@@ -1113,7 +1113,7 @@
         <v>46186</v>
       </c>
     </row>
-    <row r="22" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B22" s="10" t="s">
         <v>38</v>
       </c>
@@ -1124,7 +1124,7 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="23" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B23" s="13" t="s">
         <v>51</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>46184</v>
       </c>
     </row>
-    <row r="24" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B24" s="13" t="s">
         <v>20</v>
       </c>
@@ -1146,7 +1146,7 @@
         <v>46185</v>
       </c>
     </row>
-    <row r="25" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B25" s="13" t="s">
         <v>21</v>
       </c>
@@ -1157,7 +1157,7 @@
         <v>46185</v>
       </c>
     </row>
-    <row r="26" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="17" t="s">
         <v>49</v>
       </c>
@@ -1168,18 +1168,18 @@
         <v>46186</v>
       </c>
     </row>
-    <row r="27" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B27" s="32" t="s">
         <v>18</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D27" s="25">
         <v>46200</v>
       </c>
     </row>
-    <row r="28" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B28" s="10" t="s">
         <v>7</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>46193</v>
       </c>
     </row>
-    <row r="29" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B29" s="13" t="s">
         <v>8</v>
       </c>
@@ -1201,7 +1201,7 @@
         <v>46197</v>
       </c>
     </row>
-    <row r="30" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B30" s="13" t="s">
         <v>9</v>
       </c>
@@ -1212,25 +1212,25 @@
         <v>46199</v>
       </c>
     </row>
-    <row r="31" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B31" s="17" t="s">
         <v>56</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D31" s="15">
         <v>46200</v>
       </c>
     </row>
-    <row r="32" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="17"/>
       <c r="C32" s="18" t="s">
         <v>14</v>
       </c>
       <c r="D32" s="19"/>
     </row>
-    <row r="33" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B33" s="32" t="s">
         <v>10</v>
       </c>
@@ -1246,7 +1246,7 @@
         <v>47</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D34" s="20">
         <v>46203</v>

</xml_diff>

<commit_message>
Compleated predator class with tester. Created StaticMap class file for easear testing. Update to Prey classes to use StaticMap class. Updated Prey class tester with fix for randomness in testing
</commit_message>
<xml_diff>
--- a/documents/Milestones-for-thesis.xlsx
+++ b/documents/Milestones-for-thesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\cisc-699\final-project\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F26D26FD-4475-413E-AF1D-EA4759190F63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A66D792-B5E2-4F55-A44B-9CD707B34259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
   </bookViews>
@@ -1257,7 +1257,7 @@
         <v>28</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D35" s="15">
         <v>46212</v>
@@ -1268,7 +1268,7 @@
         <v>22</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D36" s="15">
         <v>46213</v>
@@ -1279,7 +1279,7 @@
         <v>23</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D37" s="15">
         <v>46213</v>
@@ -1290,7 +1290,7 @@
         <v>24</v>
       </c>
       <c r="C38" s="18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D38" s="19">
         <v>46214</v>

</xml_diff>

<commit_message>
update to milestone doc
</commit_message>
<xml_diff>
--- a/documents/Milestones-for-thesis.xlsx
+++ b/documents/Milestones-for-thesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\cisc-699\final-project\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A66D792-B5E2-4F55-A44B-9CD707B34259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6E9C735-8AE7-405F-AE2A-8FAC150DD7BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
   </bookViews>
@@ -1235,7 +1235,7 @@
         <v>10</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D33" s="25">
         <v>46214</v>
@@ -1301,7 +1301,7 @@
         <v>55</v>
       </c>
       <c r="C39" s="18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D39" s="19">
         <v>46214</v>

</xml_diff>

<commit_message>
Simulation v1 done + bug fixes. Documetns folder update. Read me update.
</commit_message>
<xml_diff>
--- a/documents/Milestones-for-thesis.xlsx
+++ b/documents/Milestones-for-thesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Owner\Documents\cisc-699\final-project\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB750192-150A-4C72-A5C0-4798FF54C2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{735E9C52-7372-4FBF-B7E2-6939F3D98817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6839493C-A773-4E81-BFD7-893303A98C75}"/>
   </bookViews>
@@ -1241,7 +1241,7 @@
         <v>46214</v>
       </c>
     </row>
-    <row r="34" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B34" s="10" t="s">
         <v>47</v>
       </c>
@@ -1252,7 +1252,7 @@
         <v>46203</v>
       </c>
     </row>
-    <row r="35" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B35" s="13" t="s">
         <v>28</v>
       </c>
@@ -1263,7 +1263,7 @@
         <v>46212</v>
       </c>
     </row>
-    <row r="36" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B36" s="13" t="s">
         <v>22</v>
       </c>
@@ -1274,7 +1274,7 @@
         <v>46213</v>
       </c>
     </row>
-    <row r="37" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B37" s="13" t="s">
         <v>23</v>
       </c>
@@ -1285,7 +1285,7 @@
         <v>46213</v>
       </c>
     </row>
-    <row r="38" spans="2:4" outlineLevel="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:4" hidden="1" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="B38" s="17" t="s">
         <v>24</v>
       </c>
@@ -1296,7 +1296,7 @@
         <v>46214</v>
       </c>
     </row>
-    <row r="39" spans="2:4" ht="15.75" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:4" ht="15.75" hidden="1" outlineLevel="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B39" s="17" t="s">
         <v>55</v>
       </c>
@@ -1307,7 +1307,7 @@
         <v>46214</v>
       </c>
     </row>
-    <row r="40" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:4" ht="16.5" collapsed="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B40" s="33" t="s">
         <v>36</v>
       </c>
@@ -1323,7 +1323,7 @@
         <v>33</v>
       </c>
       <c r="C41" s="11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D41" s="20">
         <v>46227</v>
@@ -1334,7 +1334,7 @@
         <v>39</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D42" s="15">
         <v>46232</v>
@@ -1345,7 +1345,7 @@
         <v>50</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D43" s="15">
         <v>46232</v>
@@ -1378,7 +1378,7 @@
         <v>25</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D46" s="15">
         <v>46234</v>
@@ -1389,7 +1389,7 @@
         <v>34</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D47" s="15">
         <v>46235</v>
@@ -1400,7 +1400,7 @@
         <v>26</v>
       </c>
       <c r="C48" s="18" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D48" s="19">
         <v>46235</v>

</xml_diff>